<commit_message>
cobranca chave mesmo sem foto
</commit_message>
<xml_diff>
--- a/LPU.xlsx
+++ b/LPU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://localiza-my.sharepoint.com/personal/caio_albanese_localiza_com/Documents/Documentos/Projetos VSCode/Agente avarias de devolucao v2/AGENTE_AVARIAS_DEVOLUCAO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://localiza-my.sharepoint.com/personal/alessandra_rodrigues_localiza_com/Documents/Documentos/Projeto_Agente_Avarias_Devolucao/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_29AD73BED340D41ADB7B2311595ED87656CC7ED3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFD869AA-DA09-481F-9EC5-B4E1C1BC9BB6}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_29AD73BED340D41ADB7B2311595ED87656CC7ED3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48D8FF9A-D494-4642-989F-82D3C2C34DA5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1191,17 +1191,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F186"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="143.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="55.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="103.6328125" customWidth="1"/>
+    <col min="3" max="3" width="55.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1221,7 +1221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>10</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>13</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>17</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>21</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>21</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>21</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>21</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>21</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>21</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>21</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>21</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>33</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>36</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>39</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>42</v>
       </c>
@@ -1479,7 +1479,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>42</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>42</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>42</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>42</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>42</v>
       </c>
@@ -1549,7 +1549,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>42</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>42</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>42</v>
       </c>
@@ -1591,7 +1591,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>42</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>42</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>42</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>42</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>57</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>57</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>62</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
         <v>62</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>62</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
         <v>62</v>
       </c>
@@ -1731,7 +1731,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
         <v>62</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
         <v>62</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B40" t="s">
         <v>70</v>
       </c>
@@ -1773,7 +1773,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>74</v>
       </c>
@@ -1787,7 +1787,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
         <v>76</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
         <v>76</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
         <v>76</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
         <v>76</v>
       </c>
@@ -1843,7 +1843,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
         <v>76</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>76</v>
       </c>
@@ -1871,7 +1871,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
         <v>76</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
         <v>76</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
         <v>76</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B51" t="s">
         <v>76</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
         <v>76</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
         <v>76</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>89</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
         <v>89</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
         <v>89</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
         <v>89</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
         <v>89</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
         <v>89</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
         <v>89</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
         <v>89</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
         <v>89</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
         <v>89</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
         <v>89</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
         <v>89</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
         <v>89</v>
       </c>
@@ -2137,7 +2137,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
         <v>104</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
         <v>104</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
         <v>104</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
         <v>104</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
         <v>109</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
         <v>109</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B73" t="s">
         <v>109</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
         <v>114</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
         <v>114</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
         <v>114</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
         <v>114</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
         <v>114</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
         <v>114</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>122</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
         <v>122</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" t="s">
         <v>126</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" t="s">
         <v>126</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" t="s">
         <v>131</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" t="s">
         <v>135</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" t="s">
         <v>137</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" t="s">
         <v>137</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" t="s">
         <v>137</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" t="s">
         <v>137</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" t="s">
         <v>137</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" t="s">
         <v>137</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" t="s">
         <v>137</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" t="s">
         <v>137</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" t="s">
         <v>137</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" t="s">
         <v>137</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" t="s">
         <v>137</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" t="s">
         <v>137</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
         <v>137</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
         <v>137</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" t="s">
         <v>137</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" t="s">
         <v>137</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B102" t="s">
         <v>137</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B103" t="s">
         <v>137</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B104" t="s">
         <v>137</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B105" t="s">
         <v>158</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B106" t="s">
         <v>158</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="107" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
         <v>158</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B108" t="s">
         <v>158</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B109" t="s">
         <v>164</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
         <v>164</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="111" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B111" t="s">
         <v>164</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="112" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
         <v>164</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="113" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B113" t="s">
         <v>164</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="114" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B114" t="s">
         <v>164</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B115" t="s">
         <v>164</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
         <v>164</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="117" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B117" t="s">
         <v>164</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="118" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B118" t="s">
         <v>164</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="119" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B119" t="s">
         <v>176</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
         <v>179</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="121" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B121" t="s">
         <v>179</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="122" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B122" t="s">
         <v>179</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
         <v>179</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="124" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B124" t="s">
         <v>179</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B125" t="s">
         <v>179</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="126" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
         <v>179</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="127" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B127" t="s">
         <v>187</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="128" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B128" t="s">
         <v>187</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="129" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B129" t="s">
         <v>191</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="130" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B130" t="s">
         <v>191</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="131" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B131" t="s">
         <v>194</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B132" t="s">
         <v>197</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="133" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B133" t="s">
         <v>197</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="134" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B134" t="s">
         <v>197</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="135" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B135" t="s">
         <v>197</v>
       </c>
@@ -3172,7 +3172,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="136" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B136" t="s">
         <v>197</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="137" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B137" t="s">
         <v>197</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="138" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B138" t="s">
         <v>197</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="139" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B139" t="s">
         <v>197</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="140" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B140" t="s">
         <v>197</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="141" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B141" t="s">
         <v>197</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="142" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B142" t="s">
         <v>197</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="143" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
         <v>197</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="144" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B144" t="s">
         <v>197</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="145" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B145" t="s">
         <v>197</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="146" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B146" t="s">
         <v>197</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="147" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B147" t="s">
         <v>197</v>
       </c>
@@ -3340,7 +3340,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="148" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B148" t="s">
         <v>197</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="149" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B149" t="s">
         <v>197</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="150" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B150" t="s">
         <v>197</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="151" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B151" t="s">
         <v>197</v>
       </c>
@@ -3396,7 +3396,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="152" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B152" t="s">
         <v>197</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="153" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B153" t="s">
         <v>220</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="154" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B154" t="s">
         <v>220</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="155" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B155" t="s">
         <v>220</v>
       </c>
@@ -3461,7 +3461,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="156" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B156" t="s">
         <v>220</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="157" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B157" t="s">
         <v>220</v>
       </c>
@@ -3495,7 +3495,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="158" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B158" t="s">
         <v>220</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="159" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B159" t="s">
         <v>220</v>
       </c>
@@ -3529,7 +3529,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="160" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B160" t="s">
         <v>220</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="161" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B161" t="s">
         <v>220</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="162" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B162" t="s">
         <v>220</v>
       </c>
@@ -3580,7 +3580,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="163" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B163" t="s">
         <v>220</v>
       </c>
@@ -3597,7 +3597,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="164" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B164" t="s">
         <v>220</v>
       </c>
@@ -3614,7 +3614,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="165" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B165" t="s">
         <v>220</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="166" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B166" t="s">
         <v>220</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="167" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B167" t="s">
         <v>220</v>
       </c>
@@ -3665,7 +3665,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="168" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B168" t="s">
         <v>220</v>
       </c>
@@ -3682,7 +3682,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="169" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B169" t="s">
         <v>220</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="170" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B170" t="s">
         <v>220</v>
       </c>
@@ -3716,7 +3716,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="171" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B171" t="s">
         <v>220</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="172" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B172" t="s">
         <v>241</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="173" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B173" t="s">
         <v>243</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="174" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B174" t="s">
         <v>245</v>
       </c>
@@ -3775,7 +3775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="175" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B175" t="s">
         <v>245</v>
       </c>
@@ -3789,7 +3789,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="176" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B176" t="s">
         <v>248</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="177" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B177" t="s">
         <v>248</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="178" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B178" t="s">
         <v>252</v>
       </c>
@@ -3834,7 +3834,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="179" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B179" t="s">
         <v>255</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B180" t="s">
         <v>258</v>
       </c>
@@ -3862,7 +3862,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="181" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B181" t="s">
         <v>260</v>
       </c>
@@ -3876,7 +3876,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="182" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B182" t="s">
         <v>74</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="183" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B183" t="s">
         <v>263</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="184" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B184" t="s">
         <v>263</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="185" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B185" t="s">
         <v>263</v>
       </c>
@@ -3932,7 +3932,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="186" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B186" t="s">
         <v>263</v>
       </c>

</xml_diff>

<commit_message>
perito de rodas analisa quatro imagens de posicoes diferentes
</commit_message>
<xml_diff>
--- a/LPU.xlsx
+++ b/LPU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://localiza-my.sharepoint.com/personal/caio_albanese_localiza_com/Documents/Documentos/Projetos VSCode/Agente avarias de devolucao v2/AGENTE_AVARIAS_DEVOLUCAO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://localiza-my.sharepoint.com/personal/alessandra_rodrigues_localiza_com/Documents/Documentos/Projeto_Agente_Avarias_Devolucao/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_29AD73BED340D41ADB7B2311595ED87656CC7ED3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFD869AA-DA09-481F-9EC5-B4E1C1BC9BB6}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_29AD73BED340D41ADB7B2311595ED87656CC7ED3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A98C4058-C64B-55B8-93B6-5F602B09A8A3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1191,17 +1191,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F186"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="143.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="55.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="143.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1221,7 +1221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>10</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>13</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>17</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>21</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>21</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>21</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>21</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>21</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>21</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>21</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>21</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>33</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>36</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>39</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>42</v>
       </c>
@@ -1479,7 +1479,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>42</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>42</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>42</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>42</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>42</v>
       </c>
@@ -1549,7 +1549,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>42</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>42</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>42</v>
       </c>
@@ -1591,7 +1591,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>42</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>42</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>42</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>42</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>57</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>57</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>62</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
         <v>62</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>62</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
         <v>62</v>
       </c>
@@ -1731,7 +1731,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
         <v>62</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
         <v>62</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B40" t="s">
         <v>70</v>
       </c>
@@ -1773,7 +1773,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>74</v>
       </c>
@@ -1787,7 +1787,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
         <v>76</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
         <v>76</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
         <v>76</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
         <v>76</v>
       </c>
@@ -1843,7 +1843,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
         <v>76</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>76</v>
       </c>
@@ -1871,7 +1871,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
         <v>76</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
         <v>76</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
         <v>76</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B51" t="s">
         <v>76</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
         <v>76</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
         <v>76</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>89</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
         <v>89</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
         <v>89</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
         <v>89</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
         <v>89</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
         <v>89</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
         <v>89</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
         <v>89</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
         <v>89</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
         <v>89</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
         <v>89</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
         <v>89</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
         <v>89</v>
       </c>
@@ -2137,7 +2137,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
         <v>104</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
         <v>104</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
         <v>104</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
         <v>104</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
         <v>109</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
         <v>109</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B73" t="s">
         <v>109</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
         <v>114</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
         <v>114</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
         <v>114</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
         <v>114</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
         <v>114</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
         <v>114</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>122</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
         <v>122</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" t="s">
         <v>126</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" t="s">
         <v>126</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" t="s">
         <v>131</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" t="s">
         <v>135</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" t="s">
         <v>137</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" t="s">
         <v>137</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" t="s">
         <v>137</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" t="s">
         <v>137</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" t="s">
         <v>137</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" t="s">
         <v>137</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" t="s">
         <v>137</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" t="s">
         <v>137</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" t="s">
         <v>137</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" t="s">
         <v>137</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" t="s">
         <v>137</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" t="s">
         <v>137</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
         <v>137</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
         <v>137</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" t="s">
         <v>137</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" t="s">
         <v>137</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B102" t="s">
         <v>137</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B103" t="s">
         <v>137</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B104" t="s">
         <v>137</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B105" t="s">
         <v>158</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B106" t="s">
         <v>158</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="107" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
         <v>158</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B108" t="s">
         <v>158</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B109" t="s">
         <v>164</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
         <v>164</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="111" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B111" t="s">
         <v>164</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="112" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
         <v>164</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="113" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B113" t="s">
         <v>164</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="114" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B114" t="s">
         <v>164</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B115" t="s">
         <v>164</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
         <v>164</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="117" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B117" t="s">
         <v>164</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="118" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B118" t="s">
         <v>164</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="119" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B119" t="s">
         <v>176</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
         <v>179</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="121" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B121" t="s">
         <v>179</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="122" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B122" t="s">
         <v>179</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
         <v>179</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="124" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B124" t="s">
         <v>179</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B125" t="s">
         <v>179</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="126" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
         <v>179</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="127" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B127" t="s">
         <v>187</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="128" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B128" t="s">
         <v>187</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="129" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B129" t="s">
         <v>191</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="130" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B130" t="s">
         <v>191</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="131" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B131" t="s">
         <v>194</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B132" t="s">
         <v>197</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="133" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B133" t="s">
         <v>197</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="134" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B134" t="s">
         <v>197</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="135" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B135" t="s">
         <v>197</v>
       </c>
@@ -3172,7 +3172,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="136" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B136" t="s">
         <v>197</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="137" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B137" t="s">
         <v>197</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="138" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B138" t="s">
         <v>197</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="139" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B139" t="s">
         <v>197</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="140" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B140" t="s">
         <v>197</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="141" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B141" t="s">
         <v>197</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="142" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B142" t="s">
         <v>197</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="143" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
         <v>197</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="144" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B144" t="s">
         <v>197</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="145" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B145" t="s">
         <v>197</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="146" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B146" t="s">
         <v>197</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="147" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B147" t="s">
         <v>197</v>
       </c>
@@ -3340,7 +3340,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="148" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B148" t="s">
         <v>197</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="149" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B149" t="s">
         <v>197</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="150" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B150" t="s">
         <v>197</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="151" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B151" t="s">
         <v>197</v>
       </c>
@@ -3396,7 +3396,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="152" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B152" t="s">
         <v>197</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="153" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B153" t="s">
         <v>220</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="154" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B154" t="s">
         <v>220</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="155" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B155" t="s">
         <v>220</v>
       </c>
@@ -3461,7 +3461,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="156" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B156" t="s">
         <v>220</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="157" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B157" t="s">
         <v>220</v>
       </c>
@@ -3495,7 +3495,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="158" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B158" t="s">
         <v>220</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="159" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B159" t="s">
         <v>220</v>
       </c>
@@ -3529,7 +3529,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="160" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B160" t="s">
         <v>220</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="161" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B161" t="s">
         <v>220</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="162" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B162" t="s">
         <v>220</v>
       </c>
@@ -3580,7 +3580,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="163" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B163" t="s">
         <v>220</v>
       </c>
@@ -3597,7 +3597,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="164" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B164" t="s">
         <v>220</v>
       </c>
@@ -3614,7 +3614,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="165" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B165" t="s">
         <v>220</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="166" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B166" t="s">
         <v>220</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="167" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B167" t="s">
         <v>220</v>
       </c>
@@ -3665,7 +3665,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="168" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B168" t="s">
         <v>220</v>
       </c>
@@ -3682,7 +3682,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="169" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B169" t="s">
         <v>220</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="170" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B170" t="s">
         <v>220</v>
       </c>
@@ -3716,7 +3716,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="171" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B171" t="s">
         <v>220</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="172" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B172" t="s">
         <v>241</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="173" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B173" t="s">
         <v>243</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="174" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B174" t="s">
         <v>245</v>
       </c>
@@ -3775,7 +3775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="175" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B175" t="s">
         <v>245</v>
       </c>
@@ -3789,7 +3789,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="176" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B176" t="s">
         <v>248</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="177" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B177" t="s">
         <v>248</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="178" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B178" t="s">
         <v>252</v>
       </c>
@@ -3834,7 +3834,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="179" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B179" t="s">
         <v>255</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B180" t="s">
         <v>258</v>
       </c>
@@ -3862,7 +3862,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="181" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B181" t="s">
         <v>260</v>
       </c>
@@ -3876,7 +3876,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="182" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B182" t="s">
         <v>74</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="183" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B183" t="s">
         <v>263</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="184" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B184" t="s">
         <v>263</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="185" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B185" t="s">
         <v>263</v>
       </c>
@@ -3932,7 +3932,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="186" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B186" t="s">
         <v>263</v>
       </c>

</xml_diff>